<commit_message>
動態表 v2_8: add Fujimoto's Scoot flights
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_24_Sep_v2_8.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_24_Sep_v2_8.xlsx
@@ -1590,11 +1590,10 @@
     <row r="2" ht="30" customHeight="1" s="123">
       <c r="A2" s="125" t="inlineStr">
         <is>
-          <t>作成: 2026/9/4（第1版・所内打合せ用ドラフト）　根拠: Gmail（ACDR2026関連スレッド）、Googleドライブ（ACDR2026事前協議チェックリスト、月次ToDo、動態表ACDR2023）、添付（ホテル部屋数検討用リスト_tt.xlsx 8/28、ACDR2026予算.xlsx 8/21、ACDR2026_Demarcation_asof0805.pptx、Draft Agenda 0805r）／v1（9/4）: 日本側サポート（中村・山口）を追記。根拠: ACDR2025動態表(as of 11/26)・荒木田9/4指示／v1_3（9/4）: 児玉修正（宮木・児玉・池田・Gerryフライト、Gerry=研究部次長）を反映し、関連セルを更新。寺坂→立部の備考取り違えを修正（児玉指摘）／v2（9/4 所内打合せ反映）: 森口=SC担当で現地参加見込、藤本=撮影主担当、宮木・児玉は内閣府に張り付かず臨機応変、27日午前に全員で会場下見、29-30日の参加者誘導、26日夜エリック長官夕食会、日本側との接続・運用テスト等を追記／v2_1（9/4）: 藤本・塩見の本人承諾を反映し「確定」に。ドレスコードとCOSEMとの役割分担を「COSEM協議事項」シートに整理／v2_2（9/6）: 宮木・児玉の10/25泊が必要と確認（25日23:40着、荒木田 9/6 WhatsApp）。JAXA登壇者＝川北氏で確定。次回COSEM合同会議は第5回（9/15オンライン、Sylvia 6/18・内閣府8/31資料）に訂正／v2_3（9/6）: WhatsApp「ACDR2026 Coordination Team」（6/15–9/2）の要点を反映。Peridot 202-205拡張（8/24）、会場無償（8/25）、コーヒーブレイクOption 1（8/26）、LTC Yong Kai（司会・モデレーター 7/30）、Field Trip帰着17:00・パレード18:00着席（8/26）、無料パス13名承認待ち、Gala挨拶枠・MOU・日本パビリオンをプログラム項目（G）として追加／v2_4（9/6）: 吉田のフライトをフィンエアー（AY1534/AY131 10/26 18:40着、AY132/AY1531 10/30 22:05発）に変更（吉田 9/6 メール）／v2_5（9/7）: 藤本・塩見を10/26夜in・10/30夜outで確定（荒木田）。Hotel Miに空きがなければ周辺ホテルを追加手配。10/31朝の見送り・清算は藤中・田中の2名で対応することを許容　【v2_6 (2026/9/9)】8/26版アジェンダ（Draft Agenda EN 0826）と突合し、27日レセプションを19:00-21:00に修正。テクニカルセッションはEOS-NTU不参加確定によりBRINへ切替（9/7）。　【v2_7 (2026/9/24)】9/17-9/24のメール・WhatsApp・9/18週次会議で更新。TSモデレーター確定（LTC Chen Yong Kai）、会場 Peridot 201-203 確定・U字28席案を9/24にCOSEMへ提案、フィールドトリップ 13:00発-16:15着、招待状v2・コンセプトノートrev1.2を池田と確認済み、Day 1 前倒しは日本パビリオン所要時間次第。　【v2_8 (2026/9/24)】森口を削除（現地不参加）。塩見のTG便（9/9発注依頼）を反映。藤本の便名はメール未確認。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>作成: 2026/9/4（第1版・所内打合せ用ドラフト）　根拠: Gmail（ACDR2026関連スレッド）、Googleドライブ（ACDR2026事前協議チェックリスト、月次ToDo、動態表ACDR2023）、添付（ホテル部屋数検討用リスト_tt.xlsx 8/28、ACDR2026予算.xlsx 8/21、ACDR2026_Demarcation_asof0805.pptx、Draft Agenda 0805r）／v1（9/4）: 日本側サポート（中村・山口）を追記。根拠: ACDR2025動態表(as of 11/26)・荒木田9/4指示／v1_3（9/4）: 児玉修正（宮木・児玉・池田・Gerryフライト、Gerry=研究部次長）を反映し、関連セルを更新。寺坂→立部の備考取り違えを修正（児玉指摘）／v2（9/4 所内打合せ反映）: 森口=SC担当で現地参加見込、藤本=撮影主担当、宮木・児玉は内閣府に張り付かず臨機応変、27日午前に全員で会場下見、29-30日の参加者誘導、26日夜エリック長官夕食会、日本側との接続・運用テスト等を追記／v2_1（9/4）: 藤本・塩見の本人承諾を反映し「確定」に。ドレスコードとCOSEMとの役割分担を「COSEM協議事項」シートに整理／v2_2（9/6）: 宮木・児玉の10/25泊が必要と確認（25日23:40着、荒木田 9/6 WhatsApp）。JAXA登壇者＝川北氏で確定。次回COSEM合同会議は第5回（9/15オンライン、Sylvia 6/18・内閣府8/31資料）に訂正／v2_3（9/6）: WhatsApp「ACDR2026 Coordination Team」（6/15–9/2）の要点を反映。Peridot 202-205拡張（8/24）、会場無償（8/25）、コーヒーブレイクOption 1（8/26）、LTC Yong Kai（司会・モデレーター 7/30）、Field Trip帰着17:00・パレード18:00着席（8/26）、無料パス13名承認待ち、Gala挨拶枠・MOU・日本パビリオンをプログラム項目（G）として追加／v2_4（9/6）: 吉田のフライトをフィンエアー（AY1534/AY131 10/26 18:40着、AY132/AY1531 10/30 22:05発）に変更（吉田 9/6 メール）／v2_5（9/7）: 藤本・塩見を10/26夜in・10/30夜outで確定（荒木田）。Hotel Miに空きがなければ周辺ホテルを追加手配。10/31朝の見送り・清算は藤中・田中の2名で対応することを許容　【v2_6 (2026/9/9)】8/26版アジェンダ（Draft Agenda EN 0826）と突合し、27日レセプションを19:00-21:00に修正。テクニカルセッションはEOS-NTU不参加確定によりBRINへ切替（9/7）。　【v2_7 (2026/9/24)】9/17-9/24のメール・WhatsApp・9/18週次会議で更新。TSモデレーター確定（LTC Chen Yong Kai）、会場 Peridot 201-203 確定・U字28席案を9/24にCOSEMへ提案、フィールドトリップ 13:00発-16:15着、招待状v2・コンセプトノートrev1.2を池田と確認済み、Day 1 前倒しは日本パビリオン所要時間次第。　【v2_8 (2026/9/24)】森口を削除（現地不参加）。塩見のTG便（9/9発注依頼）を反映。藤本はスクートTR819/TR818（WhatsApp 9/24）。</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="26.25" customHeight="1" s="123">
       <c r="A4" s="126" t="inlineStr">
         <is>
@@ -2278,22 +2277,22 @@
       </c>
       <c r="E16" s="130" t="inlineStr">
         <is>
-          <t>確定（本人承諾 9/4。便名はメール上で未確認）</t>
+          <t>確定（本人承諾 9/4。スクート便を選択 9/24）</t>
         </is>
       </c>
       <c r="F16" s="129" t="inlineStr">
         <is>
-          <t>10/26 夕方〜夜着（便名未確認。9/4に「26日夜まで着」で合意、ケイラインへ見積依頼）</t>
+          <t>10/26 TR819 関西11:30→SIN17:30</t>
         </is>
       </c>
       <c r="G16" s="129" t="inlineStr">
         <is>
-          <t>10/30 夜便・深夜便（便名未確認。9/4に「30日夜便」で合意）</t>
+          <t>11/01 TR818 SIN03:05→関西10:15（チェックイン10/31夜。藤中・田中と同便）</t>
         </is>
       </c>
       <c r="H16" s="128" t="inlineStr">
         <is>
-          <t>Hotel Mi Bencoolen 10/26-30（4泊）→要手配。Miに空きがなければ周辺ホテルを追加手配（荒木田 9/7）</t>
+          <t>Hotel Mi Bencoolen 10/26-30（4泊、31日夜は空港へ）→手配状況要確認</t>
         </is>
       </c>
       <c r="I16" s="129" t="inlineStr">
@@ -2308,7 +2307,7 @@
       </c>
       <c r="K16" s="129" t="inlineStr">
         <is>
-          <t>本人承諾済み（9/4）。26日夜in/30日夜outで確定（9/7）。本人のフライトはメール上で確認できず（9/24）→本人に便名・発券状況を確認。Hotel Miの手配状況を要確認</t>
+          <t>本人承諾済み（9/4）。フライトはスクート（TR819/TR818、108,000円＋諸税約20,650円）を本人が選択（WhatsApp 9/24 15:48-15:54）。深夜便は一人では不安のため藤中・田中と同便。ANA成田便は26日23:40着のため不採用。発券状況はケイラインへ確認</t>
         </is>
       </c>
     </row>
@@ -2363,7 +2362,7 @@
       </c>
       <c r="K17" s="129" t="inlineStr">
         <is>
-          <t>本人承諾済み（9/4）。フライトはTG便（バンコク経由）で9/9に発注依頼（塩見→藤本→ケイライン）。Eチケット控えはメール上で未確認。30日は閉会16:50後すぐ空港へ移動。Hotel Miの手配状況を要確認</t>
+          <t>本人承諾済み（9/4）。フライトはTG便（バンコク経由）で9/9に発注依頼（塩見→藤本→ケイライン）。Eチケット控えはメール上で未確認。スクート・ANA成田便は本人が希望せずTG便で確定（藤本 WhatsApp 9/24）。30日は閉会16:50後すぐ空港へ移動。Hotel Miの手配状況を要確認</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2857,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.25" customHeight="1" s="123">
       <c r="A3" s="243" t="inlineStr">
         <is>
@@ -3289,14 +3287,10 @@
       </c>
       <c r="B29" s="240" t="inlineStr">
         <is>
-          <t>Gmail: 塩見 9/9「ACDRフライトについて」（TG623/409・TG410/622、藤本→ケイライン発注）／藤本・塩見 9/4「シンガポール航空券について」</t>
-        </is>
-      </c>
-      <c r="C29" s="184" t="inlineStr">
-        <is>
-          <t>塩見・藤本のフライト。荒木田 9/24: 森口を動態表から削除</t>
-        </is>
-      </c>
+          <t>Gmail: 塩見 9/9「ACDRフライトについて」（TG623/409・TG410/622、藤本→ケイライン発注）／藤本・塩見 9/4「シンガポール航空券について」／藤本 WhatsApp 9/24: スクートTR819（10/26 関西11:30→SIN17:30）・TR818（11/1 SIN03:05→関西10:15）を選択、藤中・田中と同便</t>
+        </is>
+      </c>
+      <c r="C29" s="184" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="134" t="inlineStr">
@@ -3322,7 +3316,7 @@
     <row r="33">
       <c r="B33" s="245" t="inlineStr">
         <is>
-          <t>・時間帯別シートの担当割当は、8/6デマケと2023年の動態表を基にした『第1案』であり、所内打合せで調整する前提。</t>
+          <t>・藤本・塩見は本人承諾済み。塩見はTG便（9/9発注依頼）、藤本はスクート便（9/24選択）で手配中。Eチケットはいずれもメール上で未確認。</t>
         </is>
       </c>
     </row>
@@ -4422,12 +4416,12 @@
       <c r="E17" s="154" t="n"/>
       <c r="F17" s="164" t="inlineStr">
         <is>
-          <t>（移動）</t>
+          <t>KIX-SIN(TR819)</t>
         </is>
       </c>
       <c r="G17" s="170" t="inlineStr">
         <is>
-          <t>夕方〜夜 SIN着→Hotel Mi</t>
+          <t>SIN着17:30→Hotel Mi</t>
         </is>
       </c>
       <c r="H17" s="166" t="inlineStr">
@@ -4467,12 +4461,12 @@
       </c>
       <c r="O17" s="156" t="inlineStr">
         <is>
-          <t>Exhibition Tour誘導/閉会/夜:空港へ（便名未確認）</t>
+          <t>Exhibition Tour誘導/閉会/深夜:空港へ（藤中・田中と同行）</t>
         </is>
       </c>
       <c r="P17" s="157" t="inlineStr">
         <is>
-          <t>（10/30夜便で帰国・便名未確認）</t>
+          <t>SIN-KIX(TR818 03:05発) KIX着10:15</t>
         </is>
       </c>
       <c r="Q17" s="154" t="n"/>
@@ -4712,7 +4706,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1" s="123"/>
+    <row r="22" ht="14.25" customHeight="1" s="123">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="14.25" customHeight="1" s="123">
       <c r="A23" s="175" t="inlineStr">
         <is>
@@ -4930,9 +4930,9 @@
     <row r="29" s="123"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="F3:G3"/>
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="H3:I3"/>
@@ -4967,7 +4967,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.25" customHeight="1" s="123">
       <c r="B3" s="180" t="inlineStr">
         <is>
@@ -5873,7 +5872,6 @@
     <mergeCell ref="Y7:AD7"/>
     <mergeCell ref="Y6:AD6"/>
     <mergeCell ref="B4:K4"/>
-    <mergeCell ref="F15:K15"/>
     <mergeCell ref="N10:S10"/>
     <mergeCell ref="A23:L23"/>
     <mergeCell ref="Y13:AD13"/>
@@ -5883,9 +5881,9 @@
     <mergeCell ref="T9:X9"/>
     <mergeCell ref="T16:V16"/>
     <mergeCell ref="N24:S24"/>
+    <mergeCell ref="T12:X12"/>
     <mergeCell ref="W16:AD16"/>
     <mergeCell ref="L4:S4"/>
-    <mergeCell ref="T12:X12"/>
     <mergeCell ref="F14:K14"/>
     <mergeCell ref="N27:S27"/>
     <mergeCell ref="A21:T21"/>
@@ -5895,18 +5893,19 @@
     <mergeCell ref="T15:V15"/>
     <mergeCell ref="W18:AD18"/>
     <mergeCell ref="T17:X17"/>
-    <mergeCell ref="F16:K16"/>
-    <mergeCell ref="H10:J10"/>
     <mergeCell ref="T13:X13"/>
     <mergeCell ref="F11:K11"/>
     <mergeCell ref="Z4:AD4"/>
+    <mergeCell ref="F25:K25"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="F16:K16"/>
     <mergeCell ref="N25:S25"/>
-    <mergeCell ref="F25:K25"/>
     <mergeCell ref="D12:Q12"/>
     <mergeCell ref="W8:AD8"/>
     <mergeCell ref="Y9:AD9"/>
     <mergeCell ref="T4:Y4"/>
     <mergeCell ref="W14:AD14"/>
+    <mergeCell ref="F15:K15"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5934,7 +5933,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.25" customHeight="1" s="123">
       <c r="B3" s="180" t="inlineStr">
         <is>
@@ -7025,16 +7023,16 @@
     <mergeCell ref="W4:X4"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:L13"/>
+    <mergeCell ref="M15:R15"/>
     <mergeCell ref="V13:AC13"/>
-    <mergeCell ref="M15:R15"/>
     <mergeCell ref="S7:T7"/>
     <mergeCell ref="A23:L23"/>
     <mergeCell ref="F8:J8"/>
     <mergeCell ref="W6:AC6"/>
     <mergeCell ref="M14:R14"/>
     <mergeCell ref="S10:T10"/>
+    <mergeCell ref="S9:T9"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="S9:T9"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="N6:R6"/>
@@ -7095,8 +7093,8 @@
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="G17:J17"/>
     <mergeCell ref="M26:T26"/>
+    <mergeCell ref="G6:J6"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="G6:J6"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="G14:J14"/>
@@ -7127,7 +7125,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.25" customHeight="1" s="123">
       <c r="B3" s="180" t="inlineStr">
         <is>
@@ -8152,69 +8149,69 @@
   <mergeCells count="66">
     <mergeCell ref="M11:U11"/>
     <mergeCell ref="D11:F11"/>
+    <mergeCell ref="Y11:AD11"/>
     <mergeCell ref="N4:U4"/>
     <mergeCell ref="M10:U10"/>
+    <mergeCell ref="D27:F27"/>
     <mergeCell ref="Y14:AD14"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="Y10:AD10"/>
     <mergeCell ref="N16:U16"/>
+    <mergeCell ref="G11:K11"/>
+    <mergeCell ref="N7:U7"/>
+    <mergeCell ref="D17:F17"/>
     <mergeCell ref="G16:J16"/>
     <mergeCell ref="Y17:AD17"/>
+    <mergeCell ref="M13:U13"/>
     <mergeCell ref="G8:K8"/>
     <mergeCell ref="D16:F16"/>
+    <mergeCell ref="Y16:AD16"/>
     <mergeCell ref="G17:K17"/>
     <mergeCell ref="Y7:AD7"/>
+    <mergeCell ref="V11:X11"/>
+    <mergeCell ref="G7:K7"/>
     <mergeCell ref="Y6:AD6"/>
+    <mergeCell ref="N12:U12"/>
+    <mergeCell ref="D4:F4"/>
     <mergeCell ref="A23:L23"/>
     <mergeCell ref="D18:F18"/>
+    <mergeCell ref="Y13:AD13"/>
+    <mergeCell ref="Y18:AD18"/>
     <mergeCell ref="D9:F9"/>
     <mergeCell ref="D13:K13"/>
     <mergeCell ref="Y12:AD12"/>
     <mergeCell ref="G6:K6"/>
     <mergeCell ref="N18:U18"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="G18:K18"/>
+    <mergeCell ref="N14:U14"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="N17:U17"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="N8:U8"/>
     <mergeCell ref="L4:M4"/>
     <mergeCell ref="G24:K24"/>
     <mergeCell ref="A21:T21"/>
     <mergeCell ref="V18:X18"/>
+    <mergeCell ref="Y8:AD8"/>
+    <mergeCell ref="Y4:AA4"/>
     <mergeCell ref="G10:J10"/>
+    <mergeCell ref="D10:F10"/>
     <mergeCell ref="G26:K26"/>
+    <mergeCell ref="D12:K12"/>
+    <mergeCell ref="N9:U9"/>
+    <mergeCell ref="N25:S25"/>
     <mergeCell ref="N24:O24"/>
     <mergeCell ref="N6:U6"/>
+    <mergeCell ref="Y15:AD15"/>
     <mergeCell ref="N15:U15"/>
     <mergeCell ref="G25:K25"/>
     <mergeCell ref="Y9:AD9"/>
     <mergeCell ref="V13:X13"/>
+    <mergeCell ref="AB4:AD4"/>
     <mergeCell ref="G15:J15"/>
     <mergeCell ref="G9:K9"/>
-    <mergeCell ref="Y11:AD11"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="Y10:AD10"/>
-    <mergeCell ref="G11:K11"/>
-    <mergeCell ref="N7:U7"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="M13:U13"/>
-    <mergeCell ref="Y16:AD16"/>
-    <mergeCell ref="V11:X11"/>
-    <mergeCell ref="G7:K7"/>
-    <mergeCell ref="N12:U12"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="Y13:AD13"/>
-    <mergeCell ref="Y18:AD18"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G18:K18"/>
-    <mergeCell ref="N14:U14"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="N17:U17"/>
-    <mergeCell ref="Y8:AD8"/>
-    <mergeCell ref="Y4:AA4"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D12:K12"/>
-    <mergeCell ref="N9:U9"/>
-    <mergeCell ref="N25:S25"/>
-    <mergeCell ref="Y15:AD15"/>
-    <mergeCell ref="AB4:AD4"/>
     <mergeCell ref="G14:J14"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -8243,7 +8240,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="14.25" customHeight="1" s="123">
       <c r="B3" s="180" t="inlineStr">
         <is>
@@ -8385,7 +8381,7 @@
       </c>
       <c r="V4" s="182" t="inlineStr">
         <is>
-          <t>出発: 藤本(夜便・便名未確認)・塩見21:00(TG410)/荒木田22:20/北本23:55/吉田22:05/アゼルバイジャン23:15/インドネシア22:40/モンゴル23:55、三浦・韓国は10/31 01:20-01:35</t>
+          <t>出発: 藤本 11/1 03:05(TR818、藤中・田中と同便)・塩見21:00(TG410)/荒木田22:20/北本23:55/吉田22:05/アゼルバイジャン23:15/インドネシア22:40/モンゴル23:55、三浦・韓国は10/31 01:20-01:35</t>
         </is>
       </c>
       <c r="W4" s="183" t="n"/>
@@ -8868,7 +8864,7 @@
       <c r="T17" s="184" t="n"/>
       <c r="V17" s="190" t="inlineStr">
         <is>
-          <t>帰国準備→空港へ（30日夜便、便名未確認）</t>
+          <t>帰国準備→深夜空港へ（TR818 11/1 03:05発、藤中・田中と同便）</t>
         </is>
       </c>
       <c r="W17" s="183" t="n"/>
@@ -9122,7 +9118,6 @@
   <mergeCells count="53">
     <mergeCell ref="F24:K24"/>
     <mergeCell ref="V12:AC12"/>
-    <mergeCell ref="F12:K12"/>
     <mergeCell ref="AD6:AF6"/>
     <mergeCell ref="F18:K18"/>
     <mergeCell ref="V9:AA9"/>
@@ -9137,9 +9132,9 @@
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="F13:K13"/>
     <mergeCell ref="A23:L23"/>
+    <mergeCell ref="AC7:AF7"/>
     <mergeCell ref="O12:T12"/>
     <mergeCell ref="F9:K9"/>
-    <mergeCell ref="AC7:AF7"/>
     <mergeCell ref="AE14:AF14"/>
     <mergeCell ref="O17:T17"/>
     <mergeCell ref="O4:P4"/>
@@ -9157,13 +9152,14 @@
     <mergeCell ref="F4:K4"/>
     <mergeCell ref="O7:T7"/>
     <mergeCell ref="V17:AA17"/>
+    <mergeCell ref="F11:K11"/>
+    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="O6:T6"/>
+    <mergeCell ref="F16:K16"/>
+    <mergeCell ref="F10:K10"/>
     <mergeCell ref="AE15:AF15"/>
-    <mergeCell ref="F11:K11"/>
     <mergeCell ref="F6:K6"/>
     <mergeCell ref="O15:T15"/>
-    <mergeCell ref="F16:K16"/>
-    <mergeCell ref="O6:T6"/>
-    <mergeCell ref="F10:K10"/>
     <mergeCell ref="O18:T18"/>
     <mergeCell ref="AA10:AF10"/>
     <mergeCell ref="O9:T9"/>
@@ -9171,7 +9167,7 @@
     <mergeCell ref="O14:P14"/>
     <mergeCell ref="F7:K7"/>
     <mergeCell ref="V11:Y11"/>
-    <mergeCell ref="O10:T10"/>
+    <mergeCell ref="F12:K12"/>
     <mergeCell ref="F15:K15"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -9210,7 +9206,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="123">
       <c r="A4" s="127" t="inlineStr">
         <is>
@@ -9577,7 +9572,7 @@
       </c>
       <c r="G13" s="128" t="inlineStr">
         <is>
-          <t>10/26夕方は宮木・児玉・藤中・田中でDorsett対応（藤本・塩見は26日夜着のため入らない）。10/31朝は藤中・田中の2名で見送り・清算（荒木田 9/7: 許容。藤本・塩見は30日夜out）。COSEM送迎に空港移動を委ね、ADRCはホテルでの見送りと清算立会いに絞る。</t>
+          <t>10/26夕方は宮木・児玉・藤中・田中でDorsett対応（藤本は17:30着で夕方から合流可、塩見は19:55着）。10/31朝は藤中・田中の2名で見送り・清算（荒木田 9/7: 許容。塩見は30日夜out、藤本は31日深夜out）。COSEM送迎に空港移動を委ね、ADRCはホテルでの見送りと清算立会いに絞る。</t>
         </is>
       </c>
     </row>
@@ -9672,7 +9667,7 @@
     <row r="18" ht="43.5" customHeight="1" s="123">
       <c r="A18" s="227" t="inlineStr">
         <is>
-          <t>2. 藤本（撮影・現地一次対応）と塩見（記録・誘導）は9/4に本人承諾済み。日本側（中村・山口）と合わせ、赤字だったギャップは解消の見込み。両名は26日夜in/30日夜outで確定（9/7）。残るのは両名とMizan・森口の手配（フライト・Hotel Mi、空きなければ周辺ホテル）と、COSEMとの役割分担の合意（別シート「COSEM協議事項」）。</t>
+          <t>2. 藤本（撮影・現地一次対応）と塩見（記録・誘導）は9/4に本人承諾済み。日本側（中村・山口）と合わせ、赤字だったギャップは解消の見込み。藤本は26日17:30着（TR819）／11/1 03:05発（TR818）、塩見は26日19:55着（TG409）／30日21:00発（TG410）で手配中（9/24）。残るのは両名とMizan・森口の手配（フライト・Hotel Mi、空きなければ周辺ホテル）と、COSEMとの役割分担の合意（別シート「COSEM協議事項」）。</t>
         </is>
       </c>
     </row>
@@ -9697,7 +9692,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="123">
       <c r="A23" s="226" t="inlineStr">
         <is>
@@ -9801,7 +9795,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="123">
       <c r="A4" s="230" t="inlineStr">
         <is>
@@ -11870,7 +11863,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49" ht="15" customHeight="1" s="123">
       <c r="B49" s="237" t="inlineStr">
         <is>
@@ -11902,7 +11894,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
     <row r="54">
       <c r="B54" s="237" t="inlineStr">
         <is>
@@ -13504,7 +13495,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="242" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Assign SC admin to Fujinaka and record the Uzbekistan contact
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_24_Sep_v2_8.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_24_Sep_v2_8.xlsx
@@ -2022,12 +2022,12 @@
       </c>
       <c r="I11" s="129" t="inlineStr">
         <is>
-          <t>レセプション手配／予算管理／契約・支払／宿泊・送迎の確認／SC議案・会計報告</t>
+          <t>レセプション手配／予算管理／契約・支払／宿泊・送迎の確認／SC議案・会計報告／SC事務（議案・進行・会計報告）（9/24 荒木田）</t>
         </is>
       </c>
       <c r="J11" s="129" t="inlineStr">
         <is>
-          <t>受付デスク（会場・レセプション）、ホテル・バス・支払の現地対応、SC事務、日当支払</t>
+          <t>受付デスク（会場・レセプション）、ホテル・バス・支払の現地対応、SC事務、日当支払。SC事務（議案・進行・会計報告）を担当（森口不参加により 9/24）</t>
         </is>
       </c>
       <c r="K11" s="129" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="K12" s="166" t="inlineStr">
         <is>
-          <t>受付/SC事務(会計報告)/Gala</t>
+          <t>受付/SC事務(議案・進行・会計報告)/Gala</t>
         </is>
       </c>
       <c r="L12" s="166" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1" s="123">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="122" t="inlineStr">
         <is>
           <t>None</t>
         </is>
@@ -6435,7 +6435,7 @@
       <c r="R12" s="184" t="n"/>
       <c r="S12" s="207" t="inlineStr">
         <is>
-          <t>SC事務(会計報告)</t>
+          <t>SC事務(議案・進行・会計報告)</t>
         </is>
       </c>
       <c r="T12" s="184" t="n"/>
@@ -6907,7 +6907,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1" s="123"/>
+    <row r="22" ht="14.25" customHeight="1" s="123">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="14.25" customHeight="1" s="123">
       <c r="A23" s="200" t="inlineStr">
         <is>
@@ -8041,7 +8047,13 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1" s="123"/>
+    <row r="22" ht="14.25" customHeight="1" s="123">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
     <row r="23" ht="14.25" customHeight="1" s="123">
       <c r="A23" s="200" t="inlineStr">
         <is>
@@ -8149,8 +8161,8 @@
   <mergeCells count="66">
     <mergeCell ref="M11:U11"/>
     <mergeCell ref="D11:F11"/>
+    <mergeCell ref="N4:U4"/>
     <mergeCell ref="Y11:AD11"/>
-    <mergeCell ref="N4:U4"/>
     <mergeCell ref="M10:U10"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="Y14:AD14"/>
@@ -9660,7 +9672,7 @@
     <row r="17" ht="43.5" customHeight="1" s="123">
       <c r="A17" s="227" t="inlineStr">
         <is>
-          <t>1. 現地要員は役員3名＋運営8名（荒木田・児玉・吉田・藤中・田中・池田・Gerry・Mizan）。Mizanは会期中の参加可（フライト未取得）。森口は現地不参加（9/24 荒木田）。SC事務（議案・進行）の担当は要再割当（未手配）。</t>
+          <t>1. 現地要員は役員3名＋運営8名（荒木田・児玉・吉田・藤中・田中・池田・Gerry・Mizan）。Mizanは会期中の参加可（フライト未取得）。森口は現地不参加（9/24 荒木田）。SC事務（議案・進行・会計報告）は藤中が担当（未手配）。</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11991,7 @@
     <row r="3" ht="63.75" customHeight="1" s="123">
       <c r="A3" s="199" t="inlineStr">
         <is>
-          <t>【9/4打合せ時点の登録状況】メンバー国15か国（日本・シンガポール除く。含めると17か国でSC定足数を確保）、現地登録42名、オンライン3名。新規: バングラデシュ、パキスタン2名、PNG2名、フィジー3名、カンボジア3名、韓国3名予定（登録未）、NZ（アドバイザー）3名。ウズベキスタン2名（リソース1＋メンバー1）は回答待ち。インドネシア環境省の扱い（メンバー国か）は要確認。フィリピン・タイ・ブルネイの追加で約20か国の見込み。到着は26日と27日午前に集中させる方針だが、14時台着（バングラデシュ等）はタクシー送迎の想定。　【9/24更新】9/17以降の登録: ブルネイ1名（9/20）、韓国3名（9/21）、COSEM Fabian Tan氏（9/24）、一般オンライン1名。タイはDDPMがPrasong Thammapala氏を指名予定（9/22、ADRCは1名分負担と回答）。タジキスタン・ウズベキスタンは9/24にWhatsAppで再リマインド（両国ともビザ要）。</t>
+          <t>【9/4打合せ時点の登録状況】メンバー国15か国（日本・シンガポール除く。含めると17か国でSC定足数を確保）、現地登録42名、オンライン3名。新規: バングラデシュ、パキスタン2名、PNG2名、フィジー3名、カンボジア3名、韓国3名予定（登録未）、NZ（アドバイザー）3名。ウズベキスタン2名（リソース1＋メンバー1）は回答待ち。インドネシア環境省の扱い（メンバー国か）は要確認。フィリピン・タイ・ブルネイの追加で約20か国の見込み。到着は26日と27日午前に集中させる方針だが、14時台着（バングラデシュ等）はタクシー送迎の想定。　【9/24更新】9/17以降の登録: ブルネイ1名（9/20）、韓国3名（9/21）、COSEM Fabian Tan氏（9/24）、一般オンライン1名。タイはDDPMがPrasong Thammapala氏を指名予定（9/22、ADRCは1名分負担と回答）。タジキスタン・ウズベキスタンは9/24にWhatsAppで再リマインド（両国ともビザ要）。ウズベキスタンは連絡が取れ、2名を選出・登録予定（事務局が案内メールを再送）。</t>
         </is>
       </c>
     </row>
@@ -12699,7 +12711,7 @@
       </c>
       <c r="B18" s="241" t="inlineStr">
         <is>
-          <t>TBD ×2（1名はTSスピーカー）</t>
+          <t>TBD ×2（1名はTSスピーカー）— 2名を選出し登録予定（9/24 連絡取れた）</t>
         </is>
       </c>
       <c r="C18" s="241" t="inlineStr">
@@ -12735,7 +12747,7 @@
       <c r="I18" s="240" t="n"/>
       <c r="J18" s="240" t="inlineStr">
         <is>
-          <t>9/24 WhatsApp再リマインド。ビザ要（外交旅券のみ免除）。TS登壇者は10/2締切</t>
+          <t>9/24 WhatsApp再リマインドで連絡が取れ、2名の選出と登録を行う予定と確認。事務局からわかりやすい案内メールを再送するよう依頼済み。ビザ要（外交旅券のみ免除）、申請9/26〜。TS登壇者は10/2締切</t>
         </is>
       </c>
     </row>

</xml_diff>